<commit_message>
Synthetic Samples Metric Generation
</commit_message>
<xml_diff>
--- a/results/metrics/pipeline_per_sample.xlsx
+++ b/results/metrics/pipeline_per_sample.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2065,6 +2065,104 @@
         <v>313.4180389000103</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Synthetic_1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-05-25T12:15:13Z</t>
+        </is>
+      </c>
+      <c r="C34" t="b">
+        <v>1</v>
+      </c>
+      <c r="D34" t="b">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>3.97435089999999</v>
+      </c>
+      <c r="L34" t="n">
+        <v>5.760929100000794</v>
+      </c>
+      <c r="M34" t="n">
+        <v>1.369288800000504</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0.1629489000006288</v>
+      </c>
+      <c r="O34" t="n">
+        <v>11.83490510000047</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Synthetic_2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-05-25T12:29:21Z</t>
+        </is>
+      </c>
+      <c r="C35" t="b">
+        <v>1</v>
+      </c>
+      <c r="D35" t="b">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3.743855300001087</v>
+      </c>
+      <c r="L35" t="n">
+        <v>4.575701300000219</v>
+      </c>
+      <c r="M35" t="n">
+        <v>1.340880399999151</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.1623674000002211</v>
+      </c>
+      <c r="O35" t="n">
+        <v>10.49006420000114</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
MACS-18 Integration + Execution
</commit_message>
<xml_diff>
--- a/results/metrics/pipeline_per_sample.xlsx
+++ b/results/metrics/pipeline_per_sample.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -860,12 +860,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Normal_1</t>
+          <t>MACS_Normal_1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-26T19:06:51Z</t>
+          <t>2026-05-26T22:54:25Z</t>
         </is>
       </c>
       <c r="C8" t="b">
@@ -876,49 +876,53 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I8" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>LCA</t>
+        </is>
+      </c>
       <c r="M8" t="n">
-        <v>140.0434758999909</v>
+        <v>171.7780824999791</v>
       </c>
       <c r="N8" t="n">
-        <v>142.6225284999964</v>
+        <v>377.4370339000016</v>
       </c>
       <c r="O8" t="n">
-        <v>34.30678420000186</v>
+        <v>90.6804065000033</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1679488999943715</v>
+        <v>0.1647738000028767</v>
       </c>
       <c r="Q8" t="n">
-        <v>317.892508200006</v>
+        <v>640.8493751000206</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Normal_14</t>
+          <t>Normal_1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-26T19:51:21Z</t>
+          <t>2026-05-26T22:40:38Z</t>
         </is>
       </c>
       <c r="C9" t="b">
@@ -929,53 +933,49 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
       <c r="H9" t="n">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="I9" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="J9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>RCA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>161.7200961000053</v>
+        <v>136.3211300999974</v>
       </c>
       <c r="N9" t="n">
-        <v>401.2425762000057</v>
+        <v>155.8627302999957</v>
       </c>
       <c r="O9" t="n">
-        <v>69.84230550000211</v>
+        <v>37.18101719999686</v>
       </c>
       <c r="P9" t="n">
-        <v>0.1258051000040723</v>
+        <v>0.1587844000023324</v>
       </c>
       <c r="Q9" t="n">
-        <v>633.6039178000065</v>
+        <v>330.3014626000077</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Normal_16</t>
+          <t>Normal_14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-26T20:08:14Z</t>
+          <t>2026-05-26T19:51:21Z</t>
         </is>
       </c>
       <c r="C10" t="b">
@@ -986,19 +986,19 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="G10" t="n">
         <v>2</v>
       </c>
       <c r="H10" t="n">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="I10" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
         <v>1</v>
@@ -1009,30 +1009,30 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>138.9173406000045</v>
+        <v>161.7200961000053</v>
       </c>
       <c r="N10" t="n">
-        <v>126.4604665000079</v>
+        <v>401.2425762000057</v>
       </c>
       <c r="O10" t="n">
-        <v>30.53064630000154</v>
+        <v>69.84230550000211</v>
       </c>
       <c r="P10" t="n">
-        <v>0.1590017999988049</v>
+        <v>0.1258051000040723</v>
       </c>
       <c r="Q10" t="n">
-        <v>297.218477900009</v>
+        <v>633.6039178000065</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Normal_17</t>
+          <t>Normal_16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-26T20:13:52Z</t>
+          <t>2026-05-26T20:08:14Z</t>
         </is>
       </c>
       <c r="C11" t="b">
@@ -1043,19 +1043,19 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
       </c>
       <c r="H11" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I11" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
@@ -1066,30 +1066,30 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>147.7058454000071</v>
+        <v>138.9173406000045</v>
       </c>
       <c r="N11" t="n">
-        <v>143.0391407999996</v>
+        <v>126.4604665000079</v>
       </c>
       <c r="O11" t="n">
-        <v>35.32753480000247</v>
+        <v>30.53064630000154</v>
       </c>
       <c r="P11" t="n">
-        <v>0.1662054999906104</v>
+        <v>0.1590017999988049</v>
       </c>
       <c r="Q11" t="n">
-        <v>327.3264476999902</v>
+        <v>297.218477900009</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Normal_2</t>
+          <t>Normal_17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-26T19:19:50Z</t>
+          <t>2026-05-26T20:13:52Z</t>
         </is>
       </c>
       <c r="C12" t="b">
@@ -1100,49 +1100,53 @@
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
+        <v>17</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="n">
+        <v>15</v>
+      </c>
+      <c r="I12" t="n">
         <v>12</v>
       </c>
-      <c r="G12" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" t="n">
-        <v>10</v>
-      </c>
-      <c r="I12" t="n">
-        <v>10</v>
-      </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>RCA</t>
+        </is>
+      </c>
       <c r="M12" t="n">
-        <v>116.5343590999983</v>
+        <v>147.7058454000071</v>
       </c>
       <c r="N12" t="n">
-        <v>115.1822710999986</v>
+        <v>143.0391407999996</v>
       </c>
       <c r="O12" t="n">
-        <v>27.29071830000612</v>
+        <v>35.32753480000247</v>
       </c>
       <c r="P12" t="n">
-        <v>0.1359995999955572</v>
+        <v>0.1662054999906104</v>
       </c>
       <c r="Q12" t="n">
-        <v>259.8897338999959</v>
+        <v>327.3264476999902</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Normal_5</t>
+          <t>Normal_2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-26T19:44:53Z</t>
+          <t>2026-05-26T19:19:50Z</t>
         </is>
       </c>
       <c r="C13" t="b">
@@ -1153,42 +1157,201 @@
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
+        <v>12</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" t="n">
+        <v>10</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>116.5343590999983</v>
+      </c>
+      <c r="N13" t="n">
+        <v>115.1822710999986</v>
+      </c>
+      <c r="O13" t="n">
+        <v>27.29071830000612</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.1359995999955572</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>259.8897338999959</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Normal_5</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-05-26T22:46:30Z</t>
+        </is>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="n">
         <v>19</v>
       </c>
-      <c r="G13" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" t="n">
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="n">
         <v>17</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I14" t="n">
         <v>15</v>
       </c>
-      <c r="J13" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="inlineStr">
+      <c r="J14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>RCA</t>
         </is>
       </c>
-      <c r="M13" t="n">
-        <v>135.2277441999904</v>
-      </c>
-      <c r="N13" t="n">
-        <v>177.3040805999917</v>
-      </c>
-      <c r="O13" t="n">
-        <v>35.24707769999804</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0.1390277999889804</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>348.7659558000014</v>
+      <c r="M14" t="n">
+        <v>136.905219999986</v>
+      </c>
+      <c r="N14" t="n">
+        <v>190.1190634999948</v>
+      </c>
+      <c r="O14" t="n">
+        <v>40.92016209999565</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.2129120999888983</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>369.4821937000088</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Synthetic_1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-05-26T22:39:45Z</t>
+        </is>
+      </c>
+      <c r="C15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>4.598170100012794</v>
+      </c>
+      <c r="N15" t="n">
+        <v>14.71021489999839</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1.783923199982382</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.1607584999874234</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>21.9596237000078</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Synthetic_2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-05-26T22:39:12Z</t>
+        </is>
+      </c>
+      <c r="C16" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>4.682606799993664</v>
+      </c>
+      <c r="N16" t="n">
+        <v>12.06359209999209</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1.782922799990047</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.1681816999916919</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>19.46382969999104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>